<commit_message>
switching setup scanning order to allow more good setups
</commit_message>
<xml_diff>
--- a/Position Size Calculator.xlsx
+++ b/Position Size Calculator.xlsx
@@ -126,7 +126,7 @@
     <t>*  Symbol</t>
   </si>
   <si>
-    <t>ENRIN</t>
+    <t>PANACEABIO</t>
   </si>
   <si>
     <t>Mandatory Input Field (Not case-sensitive). It will convert to UPPER automatically</t>
@@ -135,7 +135,7 @@
     <t>* Trade Type</t>
   </si>
   <si>
-    <t>Long</t>
+    <t>Short</t>
   </si>
   <si>
     <t>Mandatory Input Field. Enter high of confirmation candle</t>
@@ -1634,10 +1634,10 @@
     <row r="16" ht="46.5" customHeight="1">
       <c r="A16" s="36" t="str">
         <f>IF(B15="Long", "*  Confirmation High", "*  Confirmation Low")</f>
-        <v>*  Confirmation High</v>
+        <v>*  Confirmation Low</v>
       </c>
       <c r="B16" s="37">
-        <v>3725.0</v>
+        <v>552.95</v>
       </c>
       <c r="C16" s="38" t="s">
         <v>29</v>
@@ -1671,7 +1671,7 @@
         <v>30</v>
       </c>
       <c r="B17" s="40">
-        <v>13.55</v>
+        <v>5.57</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>31</v>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B18" s="42">
         <f>B17/B16</f>
-        <v>0.003637583893</v>
+        <v>0.01007324351</v>
       </c>
       <c r="C18" s="43" t="s">
         <v>33</v>
@@ -1740,7 +1740,7 @@
         <v>34</v>
       </c>
       <c r="B19" s="44">
-        <v>1.8</v>
+        <v>0.25</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="7"/>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="B20" s="45">
         <f>IF(ISNUMBER(B16), IF(B15="Long", B16 + B17*B10, B16 - B17*B10), 0)</f>
-        <v>3725.6775</v>
+        <v>552.6715</v>
       </c>
       <c r="C20" s="14" t="s">
         <v>36</v>
@@ -1811,7 +1811,7 @@
    ),
    ""
 )</f>
-        <v>⚠️ WARNING: Spread exceeds limit — position sizing blocked. Avoid this trade due to high slippage risk.</v>
+        <v/>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B23" s="47">
         <f>CEILING(B17*B7, 0.1)</f>
-        <v>6.8</v>
+        <v>2.8</v>
       </c>
       <c r="C23" s="48" t="s">
         <v>39</v>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="B26" s="49">
         <f>IF(B23&gt;0,B24/B23,0)</f>
-        <v>1470.588235</v>
+        <v>3571.428571</v>
       </c>
       <c r="C26" s="48" t="s">
         <v>45</v>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B27" s="49">
         <f>IF(B20&gt;0, B25/B20, 0)</f>
-        <v>603.9170057</v>
+        <v>4071.13448</v>
       </c>
       <c r="C27" s="48" t="s">
         <v>47</v>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B28" s="49">
         <f>MIN(B26,B27)</f>
-        <v>603.9170057</v>
+        <v>3571.428571</v>
       </c>
       <c r="C28" s="48" t="s">
         <v>49</v>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="B30" s="52" t="str">
         <f>B14</f>
-        <v>ENRIN</v>
+        <v>PANACEABIO</v>
       </c>
       <c r="C30" s="53"/>
       <c r="D30" s="7"/>
@@ -2146,9 +2146,9 @@
       <c r="A31" s="54" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="55" t="str">
+      <c r="B31" s="55">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B28&gt;5, ROUND(B28/5, 0)*5, B28))</f>
-        <v>⚠️ N/A</v>
+        <v>3570</v>
       </c>
       <c r="C31" s="53" t="s">
         <v>53</v>
@@ -2181,9 +2181,9 @@
       <c r="A32" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="56" t="str">
+      <c r="B32" s="56">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",B20)</f>
-        <v>⚠️ N/A</v>
+        <v>552.6715</v>
       </c>
       <c r="C32" s="53" t="s">
         <v>55</v>
@@ -2216,9 +2216,9 @@
       <c r="A33" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="56" t="str">
+      <c r="B33" s="56">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B15="Long",CEILING(B20 - B23, 0.1),CEILING(B20 + B23, 0.1)))</f>
-        <v>⚠️ N/A</v>
+        <v>555.5</v>
       </c>
       <c r="C33" s="53" t="s">
         <v>57</v>
@@ -2251,9 +2251,9 @@
       <c r="A34" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="56" t="str">
+      <c r="B34" s="56">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B15="Long",CEILING(B32+B8*B23, 0.25),CEILING(B32-B8*B23, 0.25)))</f>
-        <v>⚠️ N/A</v>
+        <v>543</v>
       </c>
       <c r="C34" s="53" t="s">
         <v>59</v>
@@ -2286,9 +2286,9 @@
       <c r="A35" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="56" t="str">
+      <c r="B35" s="56">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B15="Long",CEILING(B32+B23*B9, 0.25),CEILING(B32-B23*B9, 0.25)))</f>
-        <v>⚠️ N/A</v>
+        <v>530.5</v>
       </c>
       <c r="C35" s="53" t="s">
         <v>61</v>
@@ -2321,9 +2321,9 @@
       <c r="A36" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="55" t="str">
+      <c r="B36" s="55">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",ROUND(B12*B31,0))</f>
-        <v>⚠️ N/A</v>
+        <v>1785</v>
       </c>
       <c r="C36" s="53" t="s">
         <v>63</v>
@@ -2356,9 +2356,9 @@
       <c r="A37" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="55" t="str">
+      <c r="B37" s="55">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",B31-B36)</f>
-        <v>⚠️ N/A</v>
+        <v>1785</v>
       </c>
       <c r="C37" s="53" t="s">
         <v>65</v>
@@ -2391,9 +2391,9 @@
       <c r="A38" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="57" t="str">
+      <c r="B38" s="57">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B15="Long",ROUND((B32-B33)*B31,0),ROUND((B33-B32)*B31,0)))</f>
-        <v>⚠️ N/A</v>
+        <v>10098</v>
       </c>
       <c r="C38" s="53" t="s">
         <v>67</v>
@@ -2426,9 +2426,9 @@
       <c r="A39" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="58" t="str">
+      <c r="B39" s="58">
         <f>IF(AND(B17&gt;0,B19&gt;0,B19/B17&gt;=B11),"⚠️ N/A",IF(B15="Long",(B34-B32)*B31,(B32-B34)*B31))</f>
-        <v>⚠️ N/A</v>
+        <v>34527.255</v>
       </c>
       <c r="C39" s="53" t="s">
         <v>69</v>

</xml_diff>